<commit_message>
- ADD: Avances con Farid
</commit_message>
<xml_diff>
--- a/seguimiento/follow-up/modelo_dominio/Modelo de Dominio Enriquecido.xlsx
+++ b/seguimiento/follow-up/modelo_dominio/Modelo de Dominio Enriquecido.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10920"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juliandiaz/Library/Mobile Documents/com~apple~CloudDocs/UCO/TalkLate/Diseño/Artefactos estrategicos/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juliandiaz/Library/Mobile Documents/com~apple~CloudDocs/UCO/TalkLate/talklate/seguimiento/follow-up/modelo_dominio/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0F1A855-BF0B-F84B-8B5B-276606B386E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="940" windowWidth="35680" windowHeight="22280" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="160" yWindow="940" windowWidth="35680" windowHeight="22280" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Modelo de dominio" sheetId="1" r:id="rId1"/>
@@ -2212,7 +2212,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="190">
+  <cellXfs count="182">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
@@ -2502,6 +2502,52 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2528,26 +2574,26 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2601,6 +2647,9 @@
     <xf numFmtId="0" fontId="9" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2610,75 +2659,6 @@
     <xf numFmtId="0" fontId="9" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3106,45 +3086,45 @@
       <c r="A2" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="125" t="s">
+      <c r="B2" s="141" t="s">
         <v>140</v>
       </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="126"/>
-      <c r="F2" s="126"/>
-      <c r="G2" s="126"/>
-      <c r="H2" s="126"/>
-      <c r="I2" s="126"/>
-      <c r="J2" s="126"/>
-      <c r="K2" s="126"/>
-      <c r="L2" s="126"/>
-      <c r="M2" s="126"/>
-      <c r="N2" s="126"/>
-      <c r="O2" s="126"/>
-      <c r="P2" s="127"/>
+      <c r="C2" s="142"/>
+      <c r="D2" s="142"/>
+      <c r="E2" s="142"/>
+      <c r="F2" s="142"/>
+      <c r="G2" s="142"/>
+      <c r="H2" s="142"/>
+      <c r="I2" s="142"/>
+      <c r="J2" s="142"/>
+      <c r="K2" s="142"/>
+      <c r="L2" s="142"/>
+      <c r="M2" s="142"/>
+      <c r="N2" s="142"/>
+      <c r="O2" s="142"/>
+      <c r="P2" s="143"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="125" t="s">
+      <c r="B3" s="141" t="s">
         <v>141</v>
       </c>
-      <c r="C3" s="126"/>
-      <c r="D3" s="126"/>
-      <c r="E3" s="126"/>
-      <c r="F3" s="126"/>
-      <c r="G3" s="126"/>
-      <c r="H3" s="126"/>
-      <c r="I3" s="126"/>
-      <c r="J3" s="126"/>
-      <c r="K3" s="126"/>
-      <c r="L3" s="126"/>
-      <c r="M3" s="126"/>
-      <c r="N3" s="126"/>
-      <c r="O3" s="126"/>
-      <c r="P3" s="127"/>
+      <c r="C3" s="142"/>
+      <c r="D3" s="142"/>
+      <c r="E3" s="142"/>
+      <c r="F3" s="142"/>
+      <c r="G3" s="142"/>
+      <c r="H3" s="142"/>
+      <c r="I3" s="142"/>
+      <c r="J3" s="142"/>
+      <c r="K3" s="142"/>
+      <c r="L3" s="142"/>
+      <c r="M3" s="142"/>
+      <c r="N3" s="142"/>
+      <c r="O3" s="142"/>
+      <c r="P3" s="143"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
@@ -3286,22 +3266,22 @@
       </c>
     </row>
     <row r="8" spans="1:16" ht="61" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="174"/>
-      <c r="B8" s="174"/>
-      <c r="C8" s="174"/>
-      <c r="D8" s="175"/>
-      <c r="E8" s="175"/>
-      <c r="F8" s="175"/>
-      <c r="G8" s="175"/>
-      <c r="H8" s="175"/>
-      <c r="I8" s="175"/>
-      <c r="J8" s="175"/>
-      <c r="K8" s="175"/>
-      <c r="L8" s="175"/>
-      <c r="M8" s="175"/>
-      <c r="N8" s="175"/>
-      <c r="O8" s="175"/>
-      <c r="P8" s="175"/>
+      <c r="A8" s="123"/>
+      <c r="B8" s="123"/>
+      <c r="C8" s="123"/>
+      <c r="D8" s="124"/>
+      <c r="E8" s="124"/>
+      <c r="F8" s="124"/>
+      <c r="G8" s="124"/>
+      <c r="H8" s="124"/>
+      <c r="I8" s="124"/>
+      <c r="J8" s="124"/>
+      <c r="K8" s="124"/>
+      <c r="L8" s="124"/>
+      <c r="M8" s="124"/>
+      <c r="N8" s="124"/>
+      <c r="O8" s="124"/>
+      <c r="P8" s="124"/>
     </row>
     <row r="9" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="107" t="s">
@@ -3326,9 +3306,9 @@
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A11" s="178"/>
-      <c r="B11" s="176"/>
-      <c r="C11" s="177"/>
+      <c r="A11" s="127"/>
+      <c r="B11" s="125"/>
+      <c r="C11" s="126"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="31" t="s">
@@ -3351,26 +3331,26 @@
       </c>
     </row>
     <row r="13" spans="1:16" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="154" t="s">
+      <c r="A13" s="170" t="s">
         <v>286</v>
       </c>
-      <c r="B13" s="155" t="s">
+      <c r="B13" s="171" t="s">
         <v>287</v>
       </c>
-      <c r="C13" s="157" t="s">
+      <c r="C13" s="173" t="s">
         <v>140</v>
       </c>
-      <c r="D13" s="156"/>
+      <c r="D13" s="172"/>
       <c r="E13" s="84" t="s">
         <v>288</v>
       </c>
       <c r="F13" s="85"/>
     </row>
     <row r="14" spans="1:16" ht="33" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="135"/>
-      <c r="B14" s="135"/>
-      <c r="C14" s="135"/>
-      <c r="D14" s="135"/>
+      <c r="A14" s="150"/>
+      <c r="B14" s="150"/>
+      <c r="C14" s="150"/>
+      <c r="D14" s="150"/>
       <c r="E14" s="84" t="s">
         <v>289</v>
       </c>
@@ -3457,45 +3437,45 @@
       <c r="A2" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="125" t="s">
+      <c r="B2" s="141" t="s">
         <v>142</v>
       </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="126"/>
-      <c r="F2" s="126"/>
-      <c r="G2" s="126"/>
-      <c r="H2" s="126"/>
-      <c r="I2" s="126"/>
-      <c r="J2" s="126"/>
-      <c r="K2" s="126"/>
-      <c r="L2" s="126"/>
-      <c r="M2" s="126"/>
-      <c r="N2" s="126"/>
-      <c r="O2" s="126"/>
-      <c r="P2" s="127"/>
+      <c r="C2" s="142"/>
+      <c r="D2" s="142"/>
+      <c r="E2" s="142"/>
+      <c r="F2" s="142"/>
+      <c r="G2" s="142"/>
+      <c r="H2" s="142"/>
+      <c r="I2" s="142"/>
+      <c r="J2" s="142"/>
+      <c r="K2" s="142"/>
+      <c r="L2" s="142"/>
+      <c r="M2" s="142"/>
+      <c r="N2" s="142"/>
+      <c r="O2" s="142"/>
+      <c r="P2" s="143"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="125" t="s">
+      <c r="B3" s="141" t="s">
         <v>143</v>
       </c>
-      <c r="C3" s="126"/>
-      <c r="D3" s="126"/>
-      <c r="E3" s="126"/>
-      <c r="F3" s="126"/>
-      <c r="G3" s="126"/>
-      <c r="H3" s="126"/>
-      <c r="I3" s="126"/>
-      <c r="J3" s="126"/>
-      <c r="K3" s="126"/>
-      <c r="L3" s="126"/>
-      <c r="M3" s="126"/>
-      <c r="N3" s="126"/>
-      <c r="O3" s="126"/>
-      <c r="P3" s="127"/>
+      <c r="C3" s="142"/>
+      <c r="D3" s="142"/>
+      <c r="E3" s="142"/>
+      <c r="F3" s="142"/>
+      <c r="G3" s="142"/>
+      <c r="H3" s="142"/>
+      <c r="I3" s="142"/>
+      <c r="J3" s="142"/>
+      <c r="K3" s="142"/>
+      <c r="L3" s="142"/>
+      <c r="M3" s="142"/>
+      <c r="N3" s="142"/>
+      <c r="O3" s="142"/>
+      <c r="P3" s="143"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
@@ -3636,65 +3616,65 @@
         <v>299</v>
       </c>
     </row>
-    <row r="8" spans="1:16" s="181" customFormat="1" ht="49" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="179" t="s">
+    <row r="8" spans="1:16" ht="49" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="128" t="s">
         <v>208</v>
       </c>
-      <c r="B8" s="180" t="s">
+      <c r="B8" s="129" t="s">
         <v>300</v>
       </c>
-      <c r="C8" s="180">
+      <c r="C8" s="129">
         <v>1</v>
       </c>
-      <c r="D8" s="180">
+      <c r="D8" s="129">
         <v>1</v>
       </c>
-      <c r="E8" s="180"/>
-      <c r="F8" s="180"/>
-      <c r="G8" s="180"/>
-      <c r="H8" s="180" t="s">
+      <c r="E8" s="129"/>
+      <c r="F8" s="129"/>
+      <c r="G8" s="129"/>
+      <c r="H8" s="129" t="s">
         <v>301</v>
       </c>
-      <c r="I8" s="180" t="s">
+      <c r="I8" s="129" t="s">
         <v>302</v>
       </c>
-      <c r="J8" s="180"/>
-      <c r="K8" s="180" t="s">
-        <v>27</v>
-      </c>
-      <c r="L8" s="180" t="s">
-        <v>27</v>
-      </c>
-      <c r="M8" s="180" t="s">
+      <c r="J8" s="129"/>
+      <c r="K8" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="L8" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="M8" s="129" t="s">
         <v>242</v>
       </c>
-      <c r="N8" s="180" t="s">
-        <v>27</v>
-      </c>
-      <c r="O8" s="180" t="s">
-        <v>27</v>
-      </c>
-      <c r="P8" s="180" t="s">
+      <c r="N8" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="O8" s="129" t="s">
+        <v>27</v>
+      </c>
+      <c r="P8" s="129" t="s">
         <v>303</v>
       </c>
     </row>
-    <row r="9" spans="1:16" s="181" customFormat="1" ht="49" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="182"/>
-      <c r="B9" s="183"/>
-      <c r="C9" s="183"/>
-      <c r="D9" s="184"/>
-      <c r="E9" s="184"/>
-      <c r="F9" s="184"/>
-      <c r="G9" s="184"/>
-      <c r="H9" s="184"/>
-      <c r="I9" s="184"/>
-      <c r="J9" s="184"/>
-      <c r="K9" s="184"/>
-      <c r="L9" s="184"/>
-      <c r="M9" s="184"/>
-      <c r="N9" s="184"/>
-      <c r="O9" s="184"/>
-      <c r="P9" s="184"/>
+    <row r="9" spans="1:16" ht="49" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="130"/>
+      <c r="B9" s="131"/>
+      <c r="C9" s="131"/>
+      <c r="D9" s="132"/>
+      <c r="E9" s="132"/>
+      <c r="F9" s="132"/>
+      <c r="G9" s="132"/>
+      <c r="H9" s="132"/>
+      <c r="I9" s="132"/>
+      <c r="J9" s="132"/>
+      <c r="K9" s="132"/>
+      <c r="L9" s="132"/>
+      <c r="M9" s="132"/>
+      <c r="N9" s="132"/>
+      <c r="O9" s="132"/>
+      <c r="P9" s="132"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="107" t="s">
@@ -3718,10 +3698,10 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:16" s="181" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="186"/>
-      <c r="B12" s="187"/>
-      <c r="C12" s="188"/>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A12" s="134"/>
+      <c r="B12" s="135"/>
+      <c r="C12" s="133"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" s="51" t="s">
@@ -3744,16 +3724,16 @@
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A14" s="159" t="s">
+      <c r="A14" s="175" t="s">
         <v>305</v>
       </c>
-      <c r="B14" s="158" t="s">
+      <c r="B14" s="174" t="s">
         <v>306</v>
       </c>
-      <c r="C14" s="160" t="s">
+      <c r="C14" s="176" t="s">
         <v>307</v>
       </c>
-      <c r="D14" s="161" t="s">
+      <c r="D14" s="177" t="s">
         <v>142</v>
       </c>
       <c r="E14" s="92" t="s">
@@ -3762,10 +3742,10 @@
       <c r="F14" s="93"/>
     </row>
     <row r="15" spans="1:16" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="135"/>
-      <c r="B15" s="146"/>
-      <c r="C15" s="135"/>
-      <c r="D15" s="135"/>
+      <c r="A15" s="150"/>
+      <c r="B15" s="162"/>
+      <c r="C15" s="150"/>
+      <c r="D15" s="150"/>
       <c r="E15" s="92" t="s">
         <v>309</v>
       </c>
@@ -3838,45 +3818,45 @@
       <c r="A2" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="125" t="s">
+      <c r="B2" s="141" t="s">
         <v>314</v>
       </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="126"/>
-      <c r="F2" s="126"/>
-      <c r="G2" s="126"/>
-      <c r="H2" s="126"/>
-      <c r="I2" s="126"/>
-      <c r="J2" s="126"/>
-      <c r="K2" s="126"/>
-      <c r="L2" s="126"/>
-      <c r="M2" s="126"/>
-      <c r="N2" s="126"/>
-      <c r="O2" s="126"/>
-      <c r="P2" s="127"/>
+      <c r="C2" s="142"/>
+      <c r="D2" s="142"/>
+      <c r="E2" s="142"/>
+      <c r="F2" s="142"/>
+      <c r="G2" s="142"/>
+      <c r="H2" s="142"/>
+      <c r="I2" s="142"/>
+      <c r="J2" s="142"/>
+      <c r="K2" s="142"/>
+      <c r="L2" s="142"/>
+      <c r="M2" s="142"/>
+      <c r="N2" s="142"/>
+      <c r="O2" s="142"/>
+      <c r="P2" s="143"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="125" t="s">
+      <c r="B3" s="141" t="s">
         <v>145</v>
       </c>
-      <c r="C3" s="126"/>
-      <c r="D3" s="126"/>
-      <c r="E3" s="126"/>
-      <c r="F3" s="126"/>
-      <c r="G3" s="126"/>
-      <c r="H3" s="126"/>
-      <c r="I3" s="126"/>
-      <c r="J3" s="126"/>
-      <c r="K3" s="126"/>
-      <c r="L3" s="126"/>
-      <c r="M3" s="126"/>
-      <c r="N3" s="126"/>
-      <c r="O3" s="126"/>
-      <c r="P3" s="127"/>
+      <c r="C3" s="142"/>
+      <c r="D3" s="142"/>
+      <c r="E3" s="142"/>
+      <c r="F3" s="142"/>
+      <c r="G3" s="142"/>
+      <c r="H3" s="142"/>
+      <c r="I3" s="142"/>
+      <c r="J3" s="142"/>
+      <c r="K3" s="142"/>
+      <c r="L3" s="142"/>
+      <c r="M3" s="142"/>
+      <c r="N3" s="142"/>
+      <c r="O3" s="142"/>
+      <c r="P3" s="143"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
@@ -4060,22 +4040,22 @@
       </c>
     </row>
     <row r="9" spans="1:16" ht="25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="174"/>
-      <c r="B9" s="174"/>
-      <c r="C9" s="174"/>
-      <c r="D9" s="175"/>
-      <c r="E9" s="175"/>
-      <c r="F9" s="175"/>
-      <c r="G9" s="175"/>
-      <c r="H9" s="175"/>
-      <c r="I9" s="175"/>
-      <c r="J9" s="175"/>
-      <c r="K9" s="175"/>
-      <c r="L9" s="175"/>
-      <c r="M9" s="175"/>
-      <c r="N9" s="175"/>
-      <c r="O9" s="175"/>
-      <c r="P9" s="175"/>
+      <c r="A9" s="123"/>
+      <c r="B9" s="123"/>
+      <c r="C9" s="123"/>
+      <c r="D9" s="124"/>
+      <c r="E9" s="124"/>
+      <c r="F9" s="124"/>
+      <c r="G9" s="124"/>
+      <c r="H9" s="124"/>
+      <c r="I9" s="124"/>
+      <c r="J9" s="124"/>
+      <c r="K9" s="124"/>
+      <c r="L9" s="124"/>
+      <c r="M9" s="124"/>
+      <c r="N9" s="124"/>
+      <c r="O9" s="124"/>
+      <c r="P9" s="124"/>
     </row>
     <row r="10" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="107" t="s">
@@ -4089,10 +4069,10 @@
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A11" s="165" t="s">
+      <c r="A11" s="178" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="151" t="s">
+      <c r="B11" s="167" t="s">
         <v>319</v>
       </c>
       <c r="C11" s="110" t="s">
@@ -4100,16 +4080,16 @@
       </c>
     </row>
     <row r="12" spans="1:16" ht="32" x14ac:dyDescent="0.2">
-      <c r="A12" s="152"/>
-      <c r="B12" s="152"/>
+      <c r="A12" s="168"/>
+      <c r="B12" s="168"/>
       <c r="C12" s="110" t="s">
         <v>317</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" s="113"/>
-      <c r="B13" s="189"/>
-      <c r="C13" s="185"/>
+      <c r="B13" s="136"/>
+      <c r="C13" s="133"/>
     </row>
     <row r="14" spans="1:16" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="51" t="s">
@@ -4132,14 +4112,14 @@
       </c>
     </row>
     <row r="15" spans="1:16" ht="19" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="159" t="s">
+      <c r="A15" s="175" t="s">
         <v>320</v>
       </c>
-      <c r="B15" s="158" t="s">
+      <c r="B15" s="174" t="s">
         <v>321</v>
       </c>
-      <c r="C15" s="160"/>
-      <c r="D15" s="161" t="s">
+      <c r="C15" s="176"/>
+      <c r="D15" s="177" t="s">
         <v>322</v>
       </c>
       <c r="E15" s="96" t="s">
@@ -4148,10 +4128,10 @@
       <c r="F15" s="93"/>
     </row>
     <row r="16" spans="1:16" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="135"/>
-      <c r="B16" s="146"/>
-      <c r="C16" s="135"/>
-      <c r="D16" s="135"/>
+      <c r="A16" s="150"/>
+      <c r="B16" s="162"/>
+      <c r="C16" s="150"/>
+      <c r="D16" s="150"/>
       <c r="E16" s="96" t="s">
         <v>324</v>
       </c>
@@ -4176,16 +4156,16 @@
       <c r="F17" s="93"/>
     </row>
     <row r="18" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="163" t="s">
+      <c r="A18" s="180" t="s">
         <v>328</v>
       </c>
-      <c r="B18" s="164" t="s">
+      <c r="B18" s="181" t="s">
         <v>329</v>
       </c>
-      <c r="C18" s="160" t="s">
+      <c r="C18" s="176" t="s">
         <v>307</v>
       </c>
-      <c r="D18" s="162" t="s">
+      <c r="D18" s="179" t="s">
         <v>314</v>
       </c>
       <c r="E18" s="96" t="s">
@@ -4194,10 +4174,10 @@
       <c r="F18" s="85"/>
     </row>
     <row r="19" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="135"/>
-      <c r="B19" s="135"/>
-      <c r="C19" s="135"/>
-      <c r="D19" s="134"/>
+      <c r="A19" s="150"/>
+      <c r="B19" s="150"/>
+      <c r="C19" s="150"/>
+      <c r="D19" s="152"/>
       <c r="E19" s="96" t="s">
         <v>331</v>
       </c>
@@ -4223,18 +4203,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C18:C19"/>
+    <mergeCell ref="C15:C16"/>
     <mergeCell ref="B2:P2"/>
     <mergeCell ref="B15:B16"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="B3:P3"/>
     <mergeCell ref="D15:D16"/>
     <mergeCell ref="A11:A12"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="A18:A19"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="C15:C16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" location="'Objetos de dominio'!A1" display="Volver al inicio" xr:uid="{00000000-0004-0000-0B00-000000000000}"/>
@@ -4275,45 +4255,45 @@
       <c r="A2" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="125" t="s">
+      <c r="B2" s="141" t="s">
         <v>336</v>
       </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="126"/>
-      <c r="F2" s="126"/>
-      <c r="G2" s="126"/>
-      <c r="H2" s="126"/>
-      <c r="I2" s="126"/>
-      <c r="J2" s="126"/>
-      <c r="K2" s="126"/>
-      <c r="L2" s="126"/>
-      <c r="M2" s="126"/>
-      <c r="N2" s="126"/>
-      <c r="O2" s="126"/>
-      <c r="P2" s="127"/>
+      <c r="C2" s="142"/>
+      <c r="D2" s="142"/>
+      <c r="E2" s="142"/>
+      <c r="F2" s="142"/>
+      <c r="G2" s="142"/>
+      <c r="H2" s="142"/>
+      <c r="I2" s="142"/>
+      <c r="J2" s="142"/>
+      <c r="K2" s="142"/>
+      <c r="L2" s="142"/>
+      <c r="M2" s="142"/>
+      <c r="N2" s="142"/>
+      <c r="O2" s="142"/>
+      <c r="P2" s="143"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="128" t="s">
+      <c r="B3" s="144" t="s">
         <v>337</v>
       </c>
-      <c r="C3" s="126"/>
-      <c r="D3" s="126"/>
-      <c r="E3" s="126"/>
-      <c r="F3" s="126"/>
-      <c r="G3" s="126"/>
-      <c r="H3" s="126"/>
-      <c r="I3" s="126"/>
-      <c r="J3" s="126"/>
-      <c r="K3" s="126"/>
-      <c r="L3" s="126"/>
-      <c r="M3" s="126"/>
-      <c r="N3" s="126"/>
-      <c r="O3" s="126"/>
-      <c r="P3" s="127"/>
+      <c r="C3" s="142"/>
+      <c r="D3" s="142"/>
+      <c r="E3" s="142"/>
+      <c r="F3" s="142"/>
+      <c r="G3" s="142"/>
+      <c r="H3" s="142"/>
+      <c r="I3" s="142"/>
+      <c r="J3" s="142"/>
+      <c r="K3" s="142"/>
+      <c r="L3" s="142"/>
+      <c r="M3" s="142"/>
+      <c r="N3" s="142"/>
+      <c r="O3" s="142"/>
+      <c r="P3" s="143"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
@@ -4497,22 +4477,18 @@
       </c>
     </row>
     <row r="9" spans="1:16" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="172"/>
-      <c r="B9" s="168"/>
-      <c r="C9" s="168"/>
-      <c r="D9" s="168"/>
-      <c r="E9" s="169"/>
-      <c r="F9" s="169"/>
-      <c r="G9" s="169"/>
-      <c r="H9" s="172"/>
-      <c r="I9" s="169"/>
-      <c r="J9" s="170"/>
-      <c r="K9" s="168"/>
-      <c r="L9" s="168"/>
-      <c r="M9" s="168"/>
-      <c r="N9" s="168"/>
-      <c r="O9" s="168"/>
-      <c r="P9" s="171"/>
+      <c r="A9" s="15"/>
+      <c r="B9" s="114"/>
+      <c r="C9" s="114"/>
+      <c r="D9" s="114"/>
+      <c r="H9" s="15"/>
+      <c r="J9" s="102"/>
+      <c r="K9" s="114"/>
+      <c r="L9" s="114"/>
+      <c r="M9" s="114"/>
+      <c r="N9" s="114"/>
+      <c r="O9" s="114"/>
+      <c r="P9" s="117"/>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A10" s="107" t="s">
@@ -4547,10 +4523,10 @@
         <v>339</v>
       </c>
     </row>
-    <row r="13" spans="1:16" s="181" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="186"/>
-      <c r="B13" s="187"/>
-      <c r="C13" s="188"/>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A13" s="134"/>
+      <c r="B13" s="135"/>
+      <c r="C13" s="133"/>
     </row>
     <row r="14" spans="1:16" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="51" t="s">
@@ -4573,16 +4549,16 @@
       </c>
     </row>
     <row r="15" spans="1:16" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="121" t="s">
+      <c r="A15" s="137" t="s">
         <v>345</v>
       </c>
-      <c r="B15" s="124" t="s">
+      <c r="B15" s="140" t="s">
         <v>346</v>
       </c>
-      <c r="C15" s="124" t="s">
+      <c r="C15" s="140" t="s">
         <v>314</v>
       </c>
-      <c r="D15" s="129" t="s">
+      <c r="D15" s="145" t="s">
         <v>336</v>
       </c>
       <c r="E15" s="100" t="s">
@@ -4591,20 +4567,20 @@
       <c r="F15" s="101"/>
     </row>
     <row r="16" spans="1:16" ht="46.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="122"/>
-      <c r="B16" s="122"/>
-      <c r="C16" s="122"/>
-      <c r="D16" s="122"/>
+      <c r="A16" s="138"/>
+      <c r="B16" s="138"/>
+      <c r="C16" s="138"/>
+      <c r="D16" s="138"/>
       <c r="E16" s="100" t="s">
         <v>348</v>
       </c>
       <c r="F16" s="101"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="123"/>
-      <c r="B17" s="123"/>
-      <c r="C17" s="123"/>
-      <c r="D17" s="123"/>
+      <c r="A17" s="139"/>
+      <c r="B17" s="139"/>
+      <c r="C17" s="139"/>
+      <c r="D17" s="139"/>
       <c r="E17" s="100" t="s">
         <v>349</v>
       </c>
@@ -5855,45 +5831,45 @@
       <c r="A2" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="125" t="s">
+      <c r="B2" s="141" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="126"/>
-      <c r="F2" s="126"/>
-      <c r="G2" s="126"/>
-      <c r="H2" s="126"/>
-      <c r="I2" s="126"/>
-      <c r="J2" s="126"/>
-      <c r="K2" s="126"/>
-      <c r="L2" s="126"/>
-      <c r="M2" s="126"/>
-      <c r="N2" s="126"/>
-      <c r="O2" s="126"/>
-      <c r="P2" s="127"/>
+      <c r="C2" s="142"/>
+      <c r="D2" s="142"/>
+      <c r="E2" s="142"/>
+      <c r="F2" s="142"/>
+      <c r="G2" s="142"/>
+      <c r="H2" s="142"/>
+      <c r="I2" s="142"/>
+      <c r="J2" s="142"/>
+      <c r="K2" s="142"/>
+      <c r="L2" s="142"/>
+      <c r="M2" s="142"/>
+      <c r="N2" s="142"/>
+      <c r="O2" s="142"/>
+      <c r="P2" s="143"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="125" t="s">
+      <c r="B3" s="141" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="126"/>
-      <c r="D3" s="126"/>
-      <c r="E3" s="126"/>
-      <c r="F3" s="126"/>
-      <c r="G3" s="126"/>
-      <c r="H3" s="126"/>
-      <c r="I3" s="126"/>
-      <c r="J3" s="126"/>
-      <c r="K3" s="126"/>
-      <c r="L3" s="126"/>
-      <c r="M3" s="126"/>
-      <c r="N3" s="126"/>
-      <c r="O3" s="126"/>
-      <c r="P3" s="127"/>
+      <c r="C3" s="142"/>
+      <c r="D3" s="142"/>
+      <c r="E3" s="142"/>
+      <c r="F3" s="142"/>
+      <c r="G3" s="142"/>
+      <c r="H3" s="142"/>
+      <c r="I3" s="142"/>
+      <c r="J3" s="142"/>
+      <c r="K3" s="142"/>
+      <c r="L3" s="142"/>
+      <c r="M3" s="142"/>
+      <c r="N3" s="142"/>
+      <c r="O3" s="142"/>
+      <c r="P3" s="143"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="23" t="s">
@@ -6225,16 +6201,16 @@
       </c>
     </row>
     <row r="16" spans="1:16" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="131" t="s">
+      <c r="A16" s="147" t="s">
         <v>54</v>
       </c>
-      <c r="B16" s="130" t="s">
+      <c r="B16" s="146" t="s">
         <v>55</v>
       </c>
-      <c r="C16" s="130" t="s">
+      <c r="C16" s="146" t="s">
         <v>56</v>
       </c>
-      <c r="D16" s="130" t="s">
+      <c r="D16" s="146" t="s">
         <v>57</v>
       </c>
       <c r="E16" s="71" t="s">
@@ -6251,10 +6227,10 @@
       </c>
     </row>
     <row r="17" spans="1:8" ht="76.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="122"/>
-      <c r="B17" s="122"/>
-      <c r="C17" s="122"/>
-      <c r="D17" s="122"/>
+      <c r="A17" s="138"/>
+      <c r="B17" s="138"/>
+      <c r="C17" s="138"/>
+      <c r="D17" s="138"/>
       <c r="E17" s="71" t="s">
         <v>62</v>
       </c>
@@ -6269,10 +6245,10 @@
       </c>
     </row>
     <row r="18" spans="1:8" ht="64" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="122"/>
-      <c r="B18" s="122"/>
-      <c r="C18" s="122"/>
-      <c r="D18" s="122"/>
+      <c r="A18" s="138"/>
+      <c r="B18" s="138"/>
+      <c r="C18" s="138"/>
+      <c r="D18" s="138"/>
       <c r="E18" s="71" t="s">
         <v>66</v>
       </c>
@@ -6287,10 +6263,10 @@
       </c>
     </row>
     <row r="19" spans="1:8" ht="64" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="123"/>
-      <c r="B19" s="123"/>
-      <c r="C19" s="123"/>
-      <c r="D19" s="123"/>
+      <c r="A19" s="139"/>
+      <c r="B19" s="139"/>
+      <c r="C19" s="139"/>
+      <c r="D19" s="139"/>
       <c r="E19" s="71" t="s">
         <v>70</v>
       </c>
@@ -6331,16 +6307,16 @@
       </c>
     </row>
     <row r="21" spans="1:8" ht="64" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="132" t="s">
+      <c r="A21" s="148" t="s">
         <v>82</v>
       </c>
-      <c r="B21" s="130" t="s">
+      <c r="B21" s="146" t="s">
         <v>83</v>
       </c>
-      <c r="C21" s="130" t="s">
+      <c r="C21" s="146" t="s">
         <v>35</v>
       </c>
-      <c r="D21" s="130" t="s">
+      <c r="D21" s="146" t="s">
         <v>57</v>
       </c>
       <c r="E21" s="71" t="s">
@@ -6357,10 +6333,10 @@
       </c>
     </row>
     <row r="22" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="123"/>
-      <c r="B22" s="123"/>
-      <c r="C22" s="123"/>
-      <c r="D22" s="123"/>
+      <c r="A22" s="139"/>
+      <c r="B22" s="139"/>
+      <c r="C22" s="139"/>
+      <c r="D22" s="139"/>
       <c r="E22" s="71" t="s">
         <v>88</v>
       </c>
@@ -6375,16 +6351,16 @@
       </c>
     </row>
     <row r="23" spans="1:8" ht="64" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="132" t="s">
+      <c r="A23" s="148" t="s">
         <v>92</v>
       </c>
-      <c r="B23" s="130" t="s">
+      <c r="B23" s="146" t="s">
         <v>93</v>
       </c>
-      <c r="C23" s="130" t="s">
+      <c r="C23" s="146" t="s">
         <v>94</v>
       </c>
-      <c r="D23" s="130" t="s">
+      <c r="D23" s="146" t="s">
         <v>57</v>
       </c>
       <c r="E23" s="71" t="s">
@@ -6401,10 +6377,10 @@
       </c>
     </row>
     <row r="24" spans="1:8" ht="64" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="123"/>
-      <c r="B24" s="123"/>
-      <c r="C24" s="123"/>
-      <c r="D24" s="123"/>
+      <c r="A24" s="139"/>
+      <c r="B24" s="139"/>
+      <c r="C24" s="139"/>
+      <c r="D24" s="139"/>
       <c r="E24" s="71" t="s">
         <v>99</v>
       </c>
@@ -6492,20 +6468,20 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A16:A19"/>
+    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="C16:C19"/>
     <mergeCell ref="B2:P2"/>
     <mergeCell ref="B21:B22"/>
     <mergeCell ref="B3:P3"/>
     <mergeCell ref="C23:C24"/>
     <mergeCell ref="D23:D24"/>
-    <mergeCell ref="A16:A19"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="C21:C22"/>
     <mergeCell ref="D16:D19"/>
-    <mergeCell ref="B16:B19"/>
     <mergeCell ref="D21:D22"/>
-    <mergeCell ref="C16:C19"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" location="'Objetos de dominio'!A1" display="Volver al inicio" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
@@ -6565,45 +6541,45 @@
       <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="125" t="s">
+      <c r="B2" s="141" t="s">
         <v>126</v>
       </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="126"/>
-      <c r="F2" s="126"/>
-      <c r="G2" s="126"/>
-      <c r="H2" s="126"/>
-      <c r="I2" s="126"/>
-      <c r="J2" s="126"/>
-      <c r="K2" s="126"/>
-      <c r="L2" s="126"/>
-      <c r="M2" s="126"/>
-      <c r="N2" s="126"/>
-      <c r="O2" s="126"/>
-      <c r="P2" s="127"/>
+      <c r="C2" s="142"/>
+      <c r="D2" s="142"/>
+      <c r="E2" s="142"/>
+      <c r="F2" s="142"/>
+      <c r="G2" s="142"/>
+      <c r="H2" s="142"/>
+      <c r="I2" s="142"/>
+      <c r="J2" s="142"/>
+      <c r="K2" s="142"/>
+      <c r="L2" s="142"/>
+      <c r="M2" s="142"/>
+      <c r="N2" s="142"/>
+      <c r="O2" s="142"/>
+      <c r="P2" s="143"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="125" t="s">
+      <c r="B3" s="141" t="s">
         <v>131</v>
       </c>
-      <c r="C3" s="126"/>
-      <c r="D3" s="126"/>
-      <c r="E3" s="126"/>
-      <c r="F3" s="126"/>
-      <c r="G3" s="126"/>
-      <c r="H3" s="126"/>
-      <c r="I3" s="126"/>
-      <c r="J3" s="126"/>
-      <c r="K3" s="126"/>
-      <c r="L3" s="126"/>
-      <c r="M3" s="126"/>
-      <c r="N3" s="126"/>
-      <c r="O3" s="126"/>
-      <c r="P3" s="127"/>
+      <c r="C3" s="142"/>
+      <c r="D3" s="142"/>
+      <c r="E3" s="142"/>
+      <c r="F3" s="142"/>
+      <c r="G3" s="142"/>
+      <c r="H3" s="142"/>
+      <c r="I3" s="142"/>
+      <c r="J3" s="142"/>
+      <c r="K3" s="142"/>
+      <c r="L3" s="142"/>
+      <c r="M3" s="142"/>
+      <c r="N3" s="142"/>
+      <c r="O3" s="142"/>
+      <c r="P3" s="143"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
@@ -6863,22 +6839,19 @@
       </c>
     </row>
     <row r="11" spans="1:16" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="166"/>
-      <c r="B11" s="167"/>
-      <c r="C11" s="168"/>
-      <c r="D11" s="168"/>
-      <c r="E11" s="169"/>
-      <c r="F11" s="169"/>
-      <c r="G11" s="169"/>
-      <c r="H11" s="170"/>
-      <c r="I11" s="170"/>
-      <c r="J11" s="170"/>
-      <c r="K11" s="170"/>
-      <c r="L11" s="170"/>
-      <c r="M11" s="170"/>
-      <c r="N11" s="170"/>
-      <c r="O11" s="170"/>
-      <c r="P11" s="171"/>
+      <c r="A11" s="116"/>
+      <c r="B11" s="121"/>
+      <c r="C11" s="114"/>
+      <c r="D11" s="114"/>
+      <c r="H11" s="102"/>
+      <c r="I11" s="102"/>
+      <c r="J11" s="102"/>
+      <c r="K11" s="102"/>
+      <c r="L11" s="102"/>
+      <c r="M11" s="102"/>
+      <c r="N11" s="102"/>
+      <c r="O11" s="102"/>
+      <c r="P11" s="117"/>
     </row>
     <row r="12" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" s="107" t="s">
@@ -6929,16 +6902,16 @@
       </c>
     </row>
     <row r="17" spans="1:8" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="132" t="s">
+      <c r="A17" s="148" t="s">
         <v>161</v>
       </c>
-      <c r="B17" s="130" t="s">
+      <c r="B17" s="146" t="s">
         <v>162</v>
       </c>
-      <c r="C17" s="130" t="s">
+      <c r="C17" s="146" t="s">
         <v>163</v>
       </c>
-      <c r="D17" s="130" t="s">
+      <c r="D17" s="146" t="s">
         <v>164</v>
       </c>
       <c r="E17" s="71" t="s">
@@ -6955,10 +6928,10 @@
       </c>
     </row>
     <row r="18" spans="1:8" ht="64" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="123"/>
-      <c r="B18" s="123"/>
-      <c r="C18" s="123"/>
-      <c r="D18" s="123"/>
+      <c r="A18" s="139"/>
+      <c r="B18" s="139"/>
+      <c r="C18" s="139"/>
+      <c r="D18" s="139"/>
       <c r="E18" s="71" t="s">
         <v>112</v>
       </c>
@@ -6973,16 +6946,16 @@
       </c>
     </row>
     <row r="19" spans="1:8" ht="64" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="141" t="s">
+      <c r="A19" s="156" t="s">
         <v>171</v>
       </c>
-      <c r="B19" s="137" t="s">
+      <c r="B19" s="153" t="s">
         <v>172</v>
       </c>
-      <c r="C19" s="137" t="s">
+      <c r="C19" s="153" t="s">
         <v>136</v>
       </c>
-      <c r="D19" s="137" t="s">
+      <c r="D19" s="153" t="s">
         <v>173</v>
       </c>
       <c r="E19" s="71" t="s">
@@ -6999,10 +6972,10 @@
       </c>
     </row>
     <row r="20" spans="1:8" ht="80" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="123"/>
-      <c r="B20" s="123"/>
-      <c r="C20" s="123"/>
-      <c r="D20" s="123"/>
+      <c r="A20" s="139"/>
+      <c r="B20" s="139"/>
+      <c r="C20" s="139"/>
+      <c r="D20" s="139"/>
       <c r="E20" s="71" t="s">
         <v>116</v>
       </c>
@@ -7113,16 +7086,16 @@
       </c>
     </row>
     <row r="36" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="142" t="s">
+      <c r="A36" s="158" t="s">
         <v>187</v>
       </c>
-      <c r="B36" s="133" t="s">
+      <c r="B36" s="157" t="s">
         <v>188</v>
       </c>
-      <c r="C36" s="133" t="s">
+      <c r="C36" s="157" t="s">
         <v>189</v>
       </c>
-      <c r="D36" s="139" t="s">
+      <c r="D36" s="151" t="s">
         <v>190</v>
       </c>
       <c r="E36" s="33" t="s">
@@ -7133,10 +7106,10 @@
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A37" s="134"/>
-      <c r="B37" s="134"/>
-      <c r="C37" s="134"/>
-      <c r="D37" s="134"/>
+      <c r="A37" s="152"/>
+      <c r="B37" s="152"/>
+      <c r="C37" s="152"/>
+      <c r="D37" s="152"/>
       <c r="E37" s="33" t="s">
         <v>114</v>
       </c>
@@ -7145,10 +7118,10 @@
       </c>
     </row>
     <row r="38" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="134"/>
-      <c r="B38" s="134"/>
-      <c r="C38" s="134"/>
-      <c r="D38" s="134"/>
+      <c r="A38" s="152"/>
+      <c r="B38" s="152"/>
+      <c r="C38" s="152"/>
+      <c r="D38" s="152"/>
       <c r="E38" s="44" t="s">
         <v>116</v>
       </c>
@@ -7157,10 +7130,10 @@
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A39" s="135"/>
-      <c r="B39" s="135"/>
-      <c r="C39" s="135"/>
-      <c r="D39" s="135"/>
+      <c r="A39" s="150"/>
+      <c r="B39" s="150"/>
+      <c r="C39" s="150"/>
+      <c r="D39" s="150"/>
       <c r="E39" s="49" t="s">
         <v>118</v>
       </c>
@@ -7189,20 +7162,20 @@
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A41" s="138" t="s">
+      <c r="A41" s="149" t="s">
         <v>196</v>
       </c>
-      <c r="B41" s="136"/>
-      <c r="C41" s="140"/>
-      <c r="D41" s="136"/>
+      <c r="B41" s="155"/>
+      <c r="C41" s="154"/>
+      <c r="D41" s="155"/>
       <c r="E41" s="46"/>
       <c r="F41" s="47"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A42" s="135"/>
-      <c r="B42" s="135"/>
-      <c r="C42" s="134"/>
-      <c r="D42" s="135"/>
+      <c r="A42" s="150"/>
+      <c r="B42" s="150"/>
+      <c r="C42" s="152"/>
+      <c r="D42" s="150"/>
       <c r="E42" s="46"/>
       <c r="F42" s="47"/>
     </row>
@@ -7228,6 +7201,10 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B2:P2"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C17:C18"/>
     <mergeCell ref="A41:A42"/>
     <mergeCell ref="B3:P3"/>
     <mergeCell ref="D36:D39"/>
@@ -7242,10 +7219,6 @@
     <mergeCell ref="A36:A39"/>
     <mergeCell ref="C36:C39"/>
     <mergeCell ref="D41:D42"/>
-    <mergeCell ref="B2:P2"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="C17:C18"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A1" location="'Objetos de dominio'!A1" display="Volver al inicio" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
@@ -7310,45 +7283,45 @@
       <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="125" t="s">
+      <c r="B2" s="141" t="s">
         <v>127</v>
       </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="126"/>
-      <c r="F2" s="126"/>
-      <c r="G2" s="126"/>
-      <c r="H2" s="126"/>
-      <c r="I2" s="126"/>
-      <c r="J2" s="126"/>
-      <c r="K2" s="126"/>
-      <c r="L2" s="126"/>
-      <c r="M2" s="126"/>
-      <c r="N2" s="126"/>
-      <c r="O2" s="126"/>
-      <c r="P2" s="127"/>
+      <c r="C2" s="142"/>
+      <c r="D2" s="142"/>
+      <c r="E2" s="142"/>
+      <c r="F2" s="142"/>
+      <c r="G2" s="142"/>
+      <c r="H2" s="142"/>
+      <c r="I2" s="142"/>
+      <c r="J2" s="142"/>
+      <c r="K2" s="142"/>
+      <c r="L2" s="142"/>
+      <c r="M2" s="142"/>
+      <c r="N2" s="142"/>
+      <c r="O2" s="142"/>
+      <c r="P2" s="143"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="125" t="s">
+      <c r="B3" s="141" t="s">
         <v>133</v>
       </c>
-      <c r="C3" s="126"/>
-      <c r="D3" s="126"/>
-      <c r="E3" s="126"/>
-      <c r="F3" s="126"/>
-      <c r="G3" s="126"/>
-      <c r="H3" s="126"/>
-      <c r="I3" s="126"/>
-      <c r="J3" s="126"/>
-      <c r="K3" s="126"/>
-      <c r="L3" s="126"/>
-      <c r="M3" s="126"/>
-      <c r="N3" s="126"/>
-      <c r="O3" s="126"/>
-      <c r="P3" s="127"/>
+      <c r="C3" s="142"/>
+      <c r="D3" s="142"/>
+      <c r="E3" s="142"/>
+      <c r="F3" s="142"/>
+      <c r="G3" s="142"/>
+      <c r="H3" s="142"/>
+      <c r="I3" s="142"/>
+      <c r="J3" s="142"/>
+      <c r="K3" s="142"/>
+      <c r="L3" s="142"/>
+      <c r="M3" s="142"/>
+      <c r="N3" s="142"/>
+      <c r="O3" s="142"/>
+      <c r="P3" s="143"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
@@ -7618,22 +7591,19 @@
       </c>
     </row>
     <row r="11" spans="1:16" ht="34" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="172"/>
-      <c r="B11" s="168"/>
-      <c r="C11" s="168"/>
-      <c r="D11" s="168"/>
-      <c r="E11" s="169"/>
-      <c r="F11" s="169"/>
-      <c r="G11" s="169"/>
-      <c r="H11" s="172"/>
-      <c r="I11" s="173"/>
-      <c r="J11" s="166"/>
-      <c r="K11" s="168"/>
-      <c r="L11" s="168"/>
-      <c r="M11" s="168"/>
-      <c r="N11" s="168"/>
-      <c r="O11" s="168"/>
-      <c r="P11" s="171"/>
+      <c r="A11" s="15"/>
+      <c r="B11" s="114"/>
+      <c r="C11" s="114"/>
+      <c r="D11" s="114"/>
+      <c r="H11" s="15"/>
+      <c r="I11" s="122"/>
+      <c r="J11" s="116"/>
+      <c r="K11" s="114"/>
+      <c r="L11" s="114"/>
+      <c r="M11" s="114"/>
+      <c r="N11" s="114"/>
+      <c r="O11" s="114"/>
+      <c r="P11" s="117"/>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" s="107" t="s">
@@ -7694,16 +7664,16 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="144" t="s">
+      <c r="A17" s="160" t="s">
         <v>216</v>
       </c>
-      <c r="B17" s="145" t="s">
+      <c r="B17" s="161" t="s">
         <v>217</v>
       </c>
-      <c r="C17" s="147" t="s">
+      <c r="C17" s="163" t="s">
         <v>218</v>
       </c>
-      <c r="D17" s="143" t="s">
+      <c r="D17" s="159" t="s">
         <v>190</v>
       </c>
       <c r="E17" s="76" t="s">
@@ -7714,10 +7684,10 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="135"/>
-      <c r="B18" s="146"/>
-      <c r="C18" s="135"/>
-      <c r="D18" s="135"/>
+      <c r="A18" s="150"/>
+      <c r="B18" s="162"/>
+      <c r="C18" s="150"/>
+      <c r="D18" s="150"/>
       <c r="E18" s="78" t="s">
         <v>114</v>
       </c>
@@ -7806,45 +7776,45 @@
       <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="125" t="s">
+      <c r="B2" s="141" t="s">
         <v>125</v>
       </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="126"/>
-      <c r="F2" s="126"/>
-      <c r="G2" s="126"/>
-      <c r="H2" s="126"/>
-      <c r="I2" s="126"/>
-      <c r="J2" s="126"/>
-      <c r="K2" s="126"/>
-      <c r="L2" s="126"/>
-      <c r="M2" s="126"/>
-      <c r="N2" s="126"/>
-      <c r="O2" s="126"/>
-      <c r="P2" s="127"/>
+      <c r="C2" s="142"/>
+      <c r="D2" s="142"/>
+      <c r="E2" s="142"/>
+      <c r="F2" s="142"/>
+      <c r="G2" s="142"/>
+      <c r="H2" s="142"/>
+      <c r="I2" s="142"/>
+      <c r="J2" s="142"/>
+      <c r="K2" s="142"/>
+      <c r="L2" s="142"/>
+      <c r="M2" s="142"/>
+      <c r="N2" s="142"/>
+      <c r="O2" s="142"/>
+      <c r="P2" s="143"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="125" t="s">
+      <c r="B3" s="141" t="s">
         <v>135</v>
       </c>
-      <c r="C3" s="126"/>
-      <c r="D3" s="126"/>
-      <c r="E3" s="126"/>
-      <c r="F3" s="126"/>
-      <c r="G3" s="126"/>
-      <c r="H3" s="126"/>
-      <c r="I3" s="126"/>
-      <c r="J3" s="126"/>
-      <c r="K3" s="126"/>
-      <c r="L3" s="126"/>
-      <c r="M3" s="126"/>
-      <c r="N3" s="126"/>
-      <c r="O3" s="126"/>
-      <c r="P3" s="127"/>
+      <c r="C3" s="142"/>
+      <c r="D3" s="142"/>
+      <c r="E3" s="142"/>
+      <c r="F3" s="142"/>
+      <c r="G3" s="142"/>
+      <c r="H3" s="142"/>
+      <c r="I3" s="142"/>
+      <c r="J3" s="142"/>
+      <c r="K3" s="142"/>
+      <c r="L3" s="142"/>
+      <c r="M3" s="142"/>
+      <c r="N3" s="142"/>
+      <c r="O3" s="142"/>
+      <c r="P3" s="143"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
@@ -8068,22 +8038,19 @@
       </c>
     </row>
     <row r="10" spans="1:16" ht="57" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="172"/>
-      <c r="B10" s="168"/>
-      <c r="C10" s="168"/>
-      <c r="D10" s="168"/>
-      <c r="E10" s="169"/>
-      <c r="F10" s="169"/>
-      <c r="G10" s="169"/>
-      <c r="H10" s="166"/>
-      <c r="I10" s="166"/>
-      <c r="J10" s="166"/>
-      <c r="K10" s="166"/>
-      <c r="L10" s="166"/>
-      <c r="M10" s="166"/>
-      <c r="N10" s="166"/>
-      <c r="O10" s="166"/>
-      <c r="P10" s="171"/>
+      <c r="A10" s="15"/>
+      <c r="B10" s="114"/>
+      <c r="C10" s="114"/>
+      <c r="D10" s="114"/>
+      <c r="H10" s="116"/>
+      <c r="I10" s="116"/>
+      <c r="J10" s="116"/>
+      <c r="K10" s="116"/>
+      <c r="L10" s="116"/>
+      <c r="M10" s="116"/>
+      <c r="N10" s="116"/>
+      <c r="O10" s="116"/>
+      <c r="P10" s="117"/>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A11" s="107" t="s">
@@ -8097,10 +8064,10 @@
       </c>
     </row>
     <row r="12" spans="1:16" ht="29" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="153" t="s">
+      <c r="A12" s="169" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="151" t="s">
+      <c r="B12" s="167" t="s">
         <v>231</v>
       </c>
       <c r="C12" s="110" t="s">
@@ -8108,8 +8075,8 @@
       </c>
     </row>
     <row r="13" spans="1:16" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="152"/>
-      <c r="B13" s="152"/>
+      <c r="A13" s="168"/>
+      <c r="B13" s="168"/>
       <c r="C13" s="110" t="s">
         <v>229</v>
       </c>
@@ -8140,16 +8107,16 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="148" t="s">
+      <c r="A18" s="164" t="s">
         <v>232</v>
       </c>
-      <c r="B18" s="149" t="s">
+      <c r="B18" s="165" t="s">
         <v>233</v>
       </c>
-      <c r="C18" s="149" t="s">
+      <c r="C18" s="165" t="s">
         <v>234</v>
       </c>
-      <c r="D18" s="150" t="s">
+      <c r="D18" s="166" t="s">
         <v>190</v>
       </c>
       <c r="E18" s="81" t="s">
@@ -8160,10 +8127,10 @@
       </c>
     </row>
     <row r="19" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="135"/>
-      <c r="B19" s="135"/>
-      <c r="C19" s="135"/>
-      <c r="D19" s="135"/>
+      <c r="A19" s="150"/>
+      <c r="B19" s="150"/>
+      <c r="C19" s="150"/>
+      <c r="D19" s="150"/>
       <c r="E19" s="81" t="s">
         <v>236</v>
       </c>
@@ -8265,45 +8232,45 @@
       <c r="A2" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="125" t="s">
+      <c r="B2" s="141" t="s">
         <v>136</v>
       </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="126"/>
-      <c r="F2" s="126"/>
-      <c r="G2" s="126"/>
-      <c r="H2" s="126"/>
-      <c r="I2" s="126"/>
-      <c r="J2" s="126"/>
-      <c r="K2" s="126"/>
-      <c r="L2" s="126"/>
-      <c r="M2" s="126"/>
-      <c r="N2" s="126"/>
-      <c r="O2" s="126"/>
-      <c r="P2" s="127"/>
+      <c r="C2" s="142"/>
+      <c r="D2" s="142"/>
+      <c r="E2" s="142"/>
+      <c r="F2" s="142"/>
+      <c r="G2" s="142"/>
+      <c r="H2" s="142"/>
+      <c r="I2" s="142"/>
+      <c r="J2" s="142"/>
+      <c r="K2" s="142"/>
+      <c r="L2" s="142"/>
+      <c r="M2" s="142"/>
+      <c r="N2" s="142"/>
+      <c r="O2" s="142"/>
+      <c r="P2" s="143"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="128" t="s">
+      <c r="B3" s="144" t="s">
         <v>137</v>
       </c>
-      <c r="C3" s="126"/>
-      <c r="D3" s="126"/>
-      <c r="E3" s="126"/>
-      <c r="F3" s="126"/>
-      <c r="G3" s="126"/>
-      <c r="H3" s="126"/>
-      <c r="I3" s="126"/>
-      <c r="J3" s="126"/>
-      <c r="K3" s="126"/>
-      <c r="L3" s="126"/>
-      <c r="M3" s="126"/>
-      <c r="N3" s="126"/>
-      <c r="O3" s="126"/>
-      <c r="P3" s="127"/>
+      <c r="C3" s="142"/>
+      <c r="D3" s="142"/>
+      <c r="E3" s="142"/>
+      <c r="F3" s="142"/>
+      <c r="G3" s="142"/>
+      <c r="H3" s="142"/>
+      <c r="I3" s="142"/>
+      <c r="J3" s="142"/>
+      <c r="K3" s="142"/>
+      <c r="L3" s="142"/>
+      <c r="M3" s="142"/>
+      <c r="N3" s="142"/>
+      <c r="O3" s="142"/>
+      <c r="P3" s="143"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
@@ -8605,22 +8572,22 @@
       </c>
     </row>
     <row r="12" spans="1:16" ht="49" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="174"/>
-      <c r="B12" s="174"/>
-      <c r="C12" s="174"/>
-      <c r="D12" s="175"/>
-      <c r="E12" s="175"/>
-      <c r="F12" s="175"/>
-      <c r="G12" s="175"/>
-      <c r="H12" s="175"/>
-      <c r="I12" s="175"/>
-      <c r="J12" s="175"/>
-      <c r="K12" s="175"/>
-      <c r="L12" s="175"/>
-      <c r="M12" s="175"/>
-      <c r="N12" s="175"/>
-      <c r="O12" s="175"/>
-      <c r="P12" s="175"/>
+      <c r="A12" s="123"/>
+      <c r="B12" s="123"/>
+      <c r="C12" s="123"/>
+      <c r="D12" s="124"/>
+      <c r="E12" s="124"/>
+      <c r="F12" s="124"/>
+      <c r="G12" s="124"/>
+      <c r="H12" s="124"/>
+      <c r="I12" s="124"/>
+      <c r="J12" s="124"/>
+      <c r="K12" s="124"/>
+      <c r="L12" s="124"/>
+      <c r="M12" s="124"/>
+      <c r="N12" s="124"/>
+      <c r="O12" s="124"/>
+      <c r="P12" s="124"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" s="107" t="s">
@@ -8665,16 +8632,16 @@
       </c>
     </row>
     <row r="18" spans="1:6" ht="52.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="148" t="s">
+      <c r="A18" s="164" t="s">
         <v>260</v>
       </c>
-      <c r="B18" s="149" t="s">
+      <c r="B18" s="165" t="s">
         <v>261</v>
       </c>
-      <c r="C18" s="149" t="s">
+      <c r="C18" s="165" t="s">
         <v>262</v>
       </c>
-      <c r="D18" s="150" t="s">
+      <c r="D18" s="166" t="s">
         <v>190</v>
       </c>
       <c r="E18" s="81" t="s">
@@ -8685,10 +8652,10 @@
       </c>
     </row>
     <row r="19" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="135"/>
-      <c r="B19" s="135"/>
-      <c r="C19" s="135"/>
-      <c r="D19" s="135"/>
+      <c r="A19" s="150"/>
+      <c r="B19" s="150"/>
+      <c r="C19" s="150"/>
+      <c r="D19" s="150"/>
       <c r="E19" s="81" t="s">
         <v>264</v>
       </c>
@@ -8745,45 +8712,45 @@
       <c r="A2" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="125" t="s">
+      <c r="B2" s="141" t="s">
         <v>138</v>
       </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="126"/>
-      <c r="F2" s="126"/>
-      <c r="G2" s="126"/>
-      <c r="H2" s="126"/>
-      <c r="I2" s="126"/>
-      <c r="J2" s="126"/>
-      <c r="K2" s="126"/>
-      <c r="L2" s="126"/>
-      <c r="M2" s="126"/>
-      <c r="N2" s="126"/>
-      <c r="O2" s="126"/>
-      <c r="P2" s="127"/>
+      <c r="C2" s="142"/>
+      <c r="D2" s="142"/>
+      <c r="E2" s="142"/>
+      <c r="F2" s="142"/>
+      <c r="G2" s="142"/>
+      <c r="H2" s="142"/>
+      <c r="I2" s="142"/>
+      <c r="J2" s="142"/>
+      <c r="K2" s="142"/>
+      <c r="L2" s="142"/>
+      <c r="M2" s="142"/>
+      <c r="N2" s="142"/>
+      <c r="O2" s="142"/>
+      <c r="P2" s="143"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="125" t="s">
+      <c r="B3" s="141" t="s">
         <v>139</v>
       </c>
-      <c r="C3" s="126"/>
-      <c r="D3" s="126"/>
-      <c r="E3" s="126"/>
-      <c r="F3" s="126"/>
-      <c r="G3" s="126"/>
-      <c r="H3" s="126"/>
-      <c r="I3" s="126"/>
-      <c r="J3" s="126"/>
-      <c r="K3" s="126"/>
-      <c r="L3" s="126"/>
-      <c r="M3" s="126"/>
-      <c r="N3" s="126"/>
-      <c r="O3" s="126"/>
-      <c r="P3" s="127"/>
+      <c r="C3" s="142"/>
+      <c r="D3" s="142"/>
+      <c r="E3" s="142"/>
+      <c r="F3" s="142"/>
+      <c r="G3" s="142"/>
+      <c r="H3" s="142"/>
+      <c r="I3" s="142"/>
+      <c r="J3" s="142"/>
+      <c r="K3" s="142"/>
+      <c r="L3" s="142"/>
+      <c r="M3" s="142"/>
+      <c r="N3" s="142"/>
+      <c r="O3" s="142"/>
+      <c r="P3" s="143"/>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
@@ -9091,22 +9058,22 @@
       </c>
     </row>
     <row r="12" spans="1:16" ht="61" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="174"/>
-      <c r="B12" s="174"/>
-      <c r="C12" s="174"/>
-      <c r="D12" s="175"/>
-      <c r="E12" s="175"/>
-      <c r="F12" s="175"/>
-      <c r="G12" s="175"/>
-      <c r="H12" s="175"/>
-      <c r="I12" s="175"/>
-      <c r="J12" s="175"/>
-      <c r="K12" s="175"/>
-      <c r="L12" s="175"/>
-      <c r="M12" s="175"/>
-      <c r="N12" s="175"/>
-      <c r="O12" s="175"/>
-      <c r="P12" s="175"/>
+      <c r="A12" s="123"/>
+      <c r="B12" s="123"/>
+      <c r="C12" s="123"/>
+      <c r="D12" s="124"/>
+      <c r="E12" s="124"/>
+      <c r="F12" s="124"/>
+      <c r="G12" s="124"/>
+      <c r="H12" s="124"/>
+      <c r="I12" s="124"/>
+      <c r="J12" s="124"/>
+      <c r="K12" s="124"/>
+      <c r="L12" s="124"/>
+      <c r="M12" s="124"/>
+      <c r="N12" s="124"/>
+      <c r="O12" s="124"/>
+      <c r="P12" s="124"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A13" s="107" t="s">
@@ -9151,16 +9118,16 @@
       </c>
     </row>
     <row r="19" spans="1:6" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="148" t="s">
+      <c r="A19" s="164" t="s">
         <v>277</v>
       </c>
-      <c r="B19" s="149" t="s">
+      <c r="B19" s="165" t="s">
         <v>278</v>
       </c>
-      <c r="C19" s="149" t="s">
+      <c r="C19" s="165" t="s">
         <v>279</v>
       </c>
-      <c r="D19" s="150" t="s">
+      <c r="D19" s="166" t="s">
         <v>190</v>
       </c>
       <c r="E19" s="81" t="s">
@@ -9171,10 +9138,10 @@
       </c>
     </row>
     <row r="20" spans="1:6" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="135"/>
-      <c r="B20" s="135"/>
-      <c r="C20" s="135"/>
-      <c r="D20" s="135"/>
+      <c r="A20" s="150"/>
+      <c r="B20" s="150"/>
+      <c r="C20" s="150"/>
+      <c r="D20" s="150"/>
       <c r="E20" s="81" t="s">
         <v>281</v>
       </c>

</xml_diff>